<commit_message>
Løst alle scripts med inventory cap 50 og max order 35
</commit_message>
<xml_diff>
--- a/weekday_demand_probabilities_plus10.xlsx
+++ b/weekday_demand_probabilities_plus10.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DemandProbabilities" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeekdayBaseDemand" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NoiseDistribution" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeekdayCenteredDemand" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CenteredPoissonOffset" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF8"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -562,31 +562,6 @@
           <t>demand_25</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>demand_26</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>demand_27</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>demand_28</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>demand_29</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>demand_30</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -640,52 +615,37 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>0.004038551481728736</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0450664812557408</v>
+        <v>0.02236789191021286</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1397060918927965</v>
+        <v>0.06194332185321045</v>
       </c>
       <c r="T2" t="n">
-        <v>0.2165444424338346</v>
+        <v>0.1143596108687832</v>
       </c>
       <c r="U2" t="n">
-        <v>0.2237625905149624</v>
+        <v>0.1583478275800003</v>
       </c>
       <c r="V2" t="n">
-        <v>0.1734160076490958</v>
+        <v>0.175404825594068</v>
       </c>
       <c r="W2" t="n">
-        <v>0.1075179247424394</v>
+        <v>0.1619159822182248</v>
       </c>
       <c r="X2" t="n">
-        <v>0.0555509277835937</v>
+        <v>0.1281123833341387</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.02460112516130579</v>
+        <v>0.08869528950362435</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.009532936000005992</v>
+        <v>0.05458300959687629</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.003283566844446509</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>0.001017905721778418</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>0</v>
+        <v>0.03023130605913239</v>
       </c>
     </row>
     <row r="3">
@@ -731,60 +691,45 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.06721358191961016</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0.1814766711829474</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>0.2449935060969791</v>
+        <v>0.008777072034527746</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.2204941554872812</v>
+        <v>0.04164978741274994</v>
       </c>
       <c r="R3" t="n">
-        <v>0.1488335549539148</v>
+        <v>0.09882024351077345</v>
       </c>
       <c r="S3" t="n">
-        <v>0.08037011967511401</v>
+        <v>0.1563103700986981</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0361665538538013</v>
+        <v>0.1854346660084502</v>
       </c>
       <c r="U3" t="n">
-        <v>0.01394995648646622</v>
+        <v>0.1759884022330869</v>
       </c>
       <c r="V3" t="n">
-        <v>0.004708110314182348</v>
+        <v>0.1391861186981053</v>
       </c>
       <c r="W3" t="n">
-        <v>0.001412433094254705</v>
+        <v>0.09435415090227638</v>
       </c>
       <c r="X3" t="n">
-        <v>0.0003813569354487703</v>
+        <v>0.05596727347016962</v>
       </c>
       <c r="Y3" t="n">
-        <v>0</v>
+        <v>0.02950901866101797</v>
       </c>
       <c r="Z3" t="n">
-        <v>0</v>
+        <v>0.01400289697014431</v>
       </c>
       <c r="AA3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -831,61 +776,46 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>0.004035983490109473</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>0.022356316076508</v>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>0.06191859676055975</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>0.1143275010568631</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>0.1583221138124134</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>0.1753971108635621</v>
       </c>
       <c r="T4" t="n">
-        <v>0</v>
+        <v>0.1619280347644893</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>0.1281370924376426</v>
       </c>
       <c r="V4" t="n">
-        <v>0.01662938425914923</v>
+        <v>0.08872290194821135</v>
       </c>
       <c r="W4" t="n">
-        <v>0.06818047546251182</v>
+        <v>0.05460646826066947</v>
       </c>
       <c r="X4" t="n">
-        <v>0.1397699746981492</v>
+        <v>0.03024788052897153</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.1910189654208039</v>
+        <v>0</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.195794439556324</v>
+        <v>0</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.1605514404361857</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>0.1097101509647269</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>0.06425880270791146</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>0.03293263638780461</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>0.01500264546555543</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>0.006151084640877727</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -931,61 +861,46 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0.05503533924501622</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>0.159602483810547</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>0.2314236015252932</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.2237094814744501</v>
+        <v>0.007176076426108307</v>
       </c>
       <c r="R5" t="n">
-        <v>0.1621893740689763</v>
+        <v>0.03552082122930442</v>
       </c>
       <c r="S5" t="n">
-        <v>0.09406983696000626</v>
+        <v>0.08791215880963363</v>
       </c>
       <c r="T5" t="n">
-        <v>0.04546708786400301</v>
+        <v>0.1450519704425123</v>
       </c>
       <c r="U5" t="n">
-        <v>0.01883636497222982</v>
+        <v>0.1794979876573386</v>
       </c>
       <c r="V5" t="n">
-        <v>0.006828182302433311</v>
+        <v>0.1776992203538715</v>
       </c>
       <c r="W5" t="n">
-        <v>0.002200192075228511</v>
+        <v>0.1465987322313526</v>
       </c>
       <c r="X5" t="n">
-        <v>0.0006380557018162682</v>
+        <v>0.1036640368999873</v>
       </c>
       <c r="Y5" t="n">
-        <v>0</v>
+        <v>0.06414075575539463</v>
       </c>
       <c r="Z5" t="n">
-        <v>0</v>
+        <v>0.03527666378943242</v>
       </c>
       <c r="AA5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>0</v>
+        <v>0.01746157640506424</v>
       </c>
     </row>
     <row r="6">
@@ -1037,54 +952,39 @@
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>0.005244242027665033</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.07428001934180856</v>
+        <v>0.02763769543730144</v>
       </c>
       <c r="R6" t="n">
-        <v>0.1931280502887023</v>
+        <v>0.0728267502773064</v>
       </c>
       <c r="S6" t="n">
-        <v>0.251066465375313</v>
+        <v>0.1279348240879958</v>
       </c>
       <c r="T6" t="n">
-        <v>0.2175909366586045</v>
+        <v>0.1685574238048214</v>
       </c>
       <c r="U6" t="n">
-        <v>0.141434108828093</v>
+        <v>0.1776629956527001</v>
       </c>
       <c r="V6" t="n">
-        <v>0.07354573659060834</v>
+        <v>0.1560503799031744</v>
       </c>
       <c r="W6" t="n">
-        <v>0.03186981918926361</v>
+        <v>0.1174859384523159</v>
       </c>
       <c r="X6" t="n">
-        <v>0.01183736141315506</v>
+        <v>0.07739537401166567</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.003847142459275395</v>
+        <v>0.04532017663703868</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.001111396710457336</v>
+        <v>0.02388419970801513</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.0002889631447189074</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1104,52 +1004,52 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2231302832612856</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3346954248919284</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2510215686689463</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1255107843344732</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0.04706654412542743</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0.01411996323762823</v>
+        <v>0.007360434843819656</v>
       </c>
       <c r="K7" t="n">
-        <v>0.003529990809407058</v>
+        <v>0.03624339623240476</v>
       </c>
       <c r="L7" t="n">
-        <v>0.000756426602015798</v>
+        <v>0.0892327558311361</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0001418299878779621</v>
+        <v>0.1464631820955012</v>
       </c>
       <c r="N7" t="n">
-        <v>2.363833131299369e-05</v>
+        <v>0.180299236892347</v>
       </c>
       <c r="O7" t="n">
-        <v>3.545749696949053e-06</v>
+        <v>0.1775617017675662</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>0.1457214428543725</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>0.1025063659377101</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>0.06309373895456452</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>0.03451987143628394</v>
       </c>
       <c r="T7" t="n">
-        <v>0</v>
+        <v>0.01699787315429383</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -1170,21 +1070,6 @@
         <v>0</v>
       </c>
       <c r="AA7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1210,43 +1095,43 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2018967249205256</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0.323034759872841</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2584278078982729</v>
+        <v>0.008210330898792001</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1378281642124122</v>
+        <v>0.03951655880792955</v>
       </c>
       <c r="K8" t="n">
-        <v>0.05513126568496488</v>
+        <v>0.09509716717083286</v>
       </c>
       <c r="L8" t="n">
-        <v>0.01764200501918876</v>
+        <v>0.1525684671055354</v>
       </c>
       <c r="M8" t="n">
-        <v>0.00470453467178367</v>
+        <v>0.1835791053043492</v>
       </c>
       <c r="N8" t="n">
-        <v>0.00107532221069341</v>
+        <v>0.1767143029943838</v>
       </c>
       <c r="O8" t="n">
-        <v>0.0002150644421386821</v>
+        <v>0.1417551706616212</v>
       </c>
       <c r="P8" t="n">
-        <v>3.823367860243238e-05</v>
+        <v>0.09746738776565068</v>
       </c>
       <c r="Q8" t="n">
-        <v>6.11738857638918e-06</v>
+        <v>0.05863916765314686</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>0.0313591112029433</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>0.01509323043481521</v>
       </c>
       <c r="T8" t="n">
         <v>0</v>
@@ -1270,21 +1155,6 @@
         <v>0</v>
       </c>
       <c r="AA8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1299,7 +1169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1310,17 +1180,77 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>weekday_weight</t>
+          <t>annual_demand_real_units</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>weekday_mean_before_rounding</t>
+          <t>number_of_weekdays_in_year</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>base_demand</t>
+          <t>mean_real_units_per_day</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>mean_model_units_per_day</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>base_demand_nearest_integer</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>max_noise_full_width_model_units</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>lower_demand_model_units</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>upper_demand_model_units</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>target_offset_mean_model_units</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>fitted_truncated_poisson_lambda</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>expected_offset_model_units</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>expected_total_model_units</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>expected_total_real_units</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>signed_deviation_min_from_nearest_base</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>signed_deviation_max_from_nearest_base</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1261,49 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24</v>
+        <v>1059.3</v>
       </c>
       <c r="C2" t="n">
-        <v>15.73658041603247</v>
+        <v>52</v>
       </c>
       <c r="D2" t="n">
-        <v>16</v>
+        <v>20.37115384615385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>20.37115384615385</v>
+      </c>
+      <c r="F2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H2" t="n">
+        <v>15</v>
+      </c>
+      <c r="I2" t="n">
+        <v>25</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5.371153846153849</v>
+      </c>
+      <c r="K2" t="n">
+        <v>5.538592738364226</v>
+      </c>
+      <c r="L2" t="n">
+        <v>5.37115384615385</v>
+      </c>
+      <c r="M2" t="n">
+        <v>20.37115384615385</v>
+      </c>
+      <c r="N2" t="n">
+        <v>20.37115384615385</v>
+      </c>
+      <c r="O2" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -1347,13 +1313,49 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>971.3000000000001</v>
+      </c>
+      <c r="C3" t="n">
+        <v>52</v>
+      </c>
+      <c r="D3" t="n">
+        <v>18.67884615384616</v>
+      </c>
+      <c r="E3" t="n">
+        <v>18.67884615384616</v>
+      </c>
+      <c r="F3" t="n">
         <v>19</v>
       </c>
-      <c r="C3" t="n">
-        <v>12.45812616269237</v>
-      </c>
-      <c r="D3" t="n">
-        <v>12</v>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="n">
+        <v>14</v>
+      </c>
+      <c r="I3" t="n">
+        <v>24</v>
+      </c>
+      <c r="J3" t="n">
+        <v>4.678846153846155</v>
+      </c>
+      <c r="K3" t="n">
+        <v>4.74529401706009</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4.678846153846155</v>
+      </c>
+      <c r="M3" t="n">
+        <v>18.67884615384616</v>
+      </c>
+      <c r="N3" t="n">
+        <v>18.67884615384616</v>
+      </c>
+      <c r="O3" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P3" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1363,13 +1365,49 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>30</v>
+        <v>920.7</v>
       </c>
       <c r="C4" t="n">
-        <v>19.67072552004059</v>
+        <v>53</v>
       </c>
       <c r="D4" t="n">
-        <v>20</v>
+        <v>17.37169811320755</v>
+      </c>
+      <c r="E4" t="n">
+        <v>17.37169811320755</v>
+      </c>
+      <c r="F4" t="n">
+        <v>17</v>
+      </c>
+      <c r="G4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H4" t="n">
+        <v>12</v>
+      </c>
+      <c r="I4" t="n">
+        <v>22</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5.371698113207547</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5.539248644424362</v>
+      </c>
+      <c r="L4" t="n">
+        <v>5.371698113207546</v>
+      </c>
+      <c r="M4" t="n">
+        <v>17.37169811320755</v>
+      </c>
+      <c r="N4" t="n">
+        <v>17.37169811320755</v>
+      </c>
+      <c r="O4" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P4" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -1379,13 +1417,49 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>18</v>
+        <v>1032.9</v>
       </c>
       <c r="C5" t="n">
-        <v>11.80243531202435</v>
+        <v>52</v>
       </c>
       <c r="D5" t="n">
-        <v>12</v>
+        <v>19.86346153846154</v>
+      </c>
+      <c r="E5" t="n">
+        <v>19.86346153846154</v>
+      </c>
+      <c r="F5" t="n">
+        <v>20</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" t="n">
+        <v>15</v>
+      </c>
+      <c r="I5" t="n">
+        <v>25</v>
+      </c>
+      <c r="J5" t="n">
+        <v>4.863461538461539</v>
+      </c>
+      <c r="K5" t="n">
+        <v>4.949894499460882</v>
+      </c>
+      <c r="L5" t="n">
+        <v>4.863461538461539</v>
+      </c>
+      <c r="M5" t="n">
+        <v>19.86346153846154</v>
+      </c>
+      <c r="N5" t="n">
+        <v>19.86346153846154</v>
+      </c>
+      <c r="O5" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P5" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -1395,13 +1469,49 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>23</v>
+        <v>995.5000000000001</v>
       </c>
       <c r="C6" t="n">
-        <v>15.08088956536445</v>
+        <v>52</v>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>19.14423076923077</v>
+      </c>
+      <c r="E6" t="n">
+        <v>19.14423076923077</v>
+      </c>
+      <c r="F6" t="n">
+        <v>19</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I6" t="n">
+        <v>24</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5.14423076923077</v>
+      </c>
+      <c r="K6" t="n">
+        <v>5.270102960829012</v>
+      </c>
+      <c r="L6" t="n">
+        <v>5.144230769230771</v>
+      </c>
+      <c r="M6" t="n">
+        <v>19.14423076923077</v>
+      </c>
+      <c r="N6" t="n">
+        <v>19.14423076923077</v>
+      </c>
+      <c r="O6" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P6" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -1411,13 +1521,49 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>667.7</v>
+      </c>
+      <c r="C7" t="n">
+        <v>52</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12.84038461538462</v>
+      </c>
+      <c r="E7" t="n">
+        <v>12.84038461538462</v>
+      </c>
+      <c r="F7" t="n">
+        <v>13</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" t="n">
+        <v>8</v>
+      </c>
+      <c r="I7" t="n">
+        <v>18</v>
+      </c>
+      <c r="J7" t="n">
+        <v>4.840384615384616</v>
+      </c>
+      <c r="K7" t="n">
+        <v>4.924083563192912</v>
+      </c>
+      <c r="L7" t="n">
+        <v>4.840384615384616</v>
+      </c>
+      <c r="M7" t="n">
+        <v>12.84038461538461</v>
+      </c>
+      <c r="N7" t="n">
+        <v>12.84038461538461</v>
+      </c>
+      <c r="O7" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P7" t="n">
         <v>5</v>
-      </c>
-      <c r="C7" t="n">
-        <v>3.278454253340099</v>
-      </c>
-      <c r="D7" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1427,12 +1573,48 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>610.5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>52</v>
+      </c>
+      <c r="D8" t="n">
+        <v>11.74038461538461</v>
+      </c>
+      <c r="E8" t="n">
+        <v>11.74038461538461</v>
+      </c>
+      <c r="F8" t="n">
+        <v>12</v>
+      </c>
+      <c r="G8" t="n">
+        <v>10</v>
+      </c>
+      <c r="H8" t="n">
         <v>7</v>
       </c>
-      <c r="C8" t="n">
-        <v>4.589835954676138</v>
-      </c>
-      <c r="D8" t="n">
+      <c r="I8" t="n">
+        <v>17</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4.740384615384615</v>
+      </c>
+      <c r="K8" t="n">
+        <v>4.813028767664369</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4.740384615384616</v>
+      </c>
+      <c r="M8" t="n">
+        <v>11.74038461538462</v>
+      </c>
+      <c r="N8" t="n">
+        <v>11.74038461538462</v>
+      </c>
+      <c r="O8" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P8" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1447,7 +1629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:BI8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1458,62 +1640,302 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>noise_lambda</t>
+          <t>lower_demand_model_units</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_0</t>
+          <t>upper_demand_model_units</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_1</t>
+          <t>target_offset_mean_model_units</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_2</t>
+          <t>fitted_truncated_poisson_lambda</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_3</t>
+          <t>expected_total_model_units</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_4</t>
+          <t>P_offset_0_demand_15</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_5</t>
+          <t>P_offset_1_demand_16</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_6</t>
+          <t>P_offset_2_demand_17</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_7</t>
+          <t>P_offset_3_demand_18</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_8</t>
+          <t>P_offset_4_demand_19</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_9</t>
+          <t>P_offset_5_demand_20</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_10</t>
+          <t>P_offset_6_demand_21</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_7_demand_22</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_8_demand_23</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_9_demand_24</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_10_demand_25</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_0_demand_14</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_1_demand_15</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_2_demand_16</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_3_demand_17</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_4_demand_18</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_5_demand_19</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_6_demand_20</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_7_demand_21</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_8_demand_22</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_9_demand_23</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_10_demand_24</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_0_demand_12</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_1_demand_13</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_2_demand_14</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_3_demand_15</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_4_demand_16</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_5_demand_17</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_6_demand_18</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_7_demand_19</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_8_demand_20</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_9_demand_21</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_10_demand_22</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_0_demand_8</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_1_demand_9</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_2_demand_10</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_3_demand_11</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_4_demand_12</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_5_demand_13</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_6_demand_14</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_7_demand_15</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_8_demand_16</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_9_demand_17</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_10_demand_18</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_0_demand_7</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_1_demand_8</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_2_demand_9</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_3_demand_10</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_4_demand_11</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_5_demand_12</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_6_demand_13</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_7_demand_14</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_8_demand_15</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_9_demand_16</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_10_demand_17</t>
         </is>
       </c>
     </row>
@@ -1524,41 +1946,97 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.1</v>
+        <v>15</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0450664812557408</v>
+        <v>25</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1397060918927965</v>
+        <v>5.371153846153849</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2165444424338346</v>
+        <v>5.538592738364226</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2237625905149624</v>
+        <v>20.37115384615385</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1734160076490958</v>
+        <v>0.004038551481728736</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1075179247424394</v>
+        <v>0.02236789191021286</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0555509277835937</v>
+        <v>0.06194332185321045</v>
       </c>
       <c r="J2" t="n">
-        <v>0.02460112516130579</v>
+        <v>0.1143596108687832</v>
       </c>
       <c r="K2" t="n">
-        <v>0.009532936000005992</v>
+        <v>0.1583478275800003</v>
       </c>
       <c r="L2" t="n">
-        <v>0.003283566844446509</v>
+        <v>0.175404825594068</v>
       </c>
       <c r="M2" t="n">
-        <v>0.001017905721778418</v>
-      </c>
+        <v>0.1619159822182248</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.1281123833341387</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.08869528950362435</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.05458300959687629</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.03023130605913239</v>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
+      <c r="BI2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1567,41 +2045,97 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.7</v>
+        <v>14</v>
       </c>
       <c r="C3" t="n">
-        <v>0.06721358191961016</v>
+        <v>24</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1814766711829474</v>
+        <v>4.678846153846155</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2449935060969791</v>
+        <v>4.74529401706009</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2204941554872812</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.1488335549539148</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.08037011967511401</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.0361665538538013</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.01394995648646622</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.004708110314182348</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.001412433094254705</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.0003813569354487703</v>
-      </c>
+        <v>18.67884615384616</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="n">
+        <v>0.008777072034527746</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.04164978741274994</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.09882024351077345</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.1563103700986981</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.1854346660084502</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.1759884022330869</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0.1391861186981053</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.09435415090227638</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0.05596727347016962</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0.02950901866101797</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0.01400289697014431</v>
+      </c>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr"/>
+      <c r="BG3" t="inlineStr"/>
+      <c r="BH3" t="inlineStr"/>
+      <c r="BI3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1610,41 +2144,97 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4.1</v>
+        <v>12</v>
       </c>
       <c r="C4" t="n">
-        <v>0.01662938425914923</v>
+        <v>22</v>
       </c>
       <c r="D4" t="n">
-        <v>0.06818047546251182</v>
+        <v>5.371698113207547</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1397699746981492</v>
+        <v>5.539248644424362</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1910189654208039</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.195794439556324</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.1605514404361857</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.1097101509647269</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.06425880270791146</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.03293263638780461</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.01500264546555543</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.006151084640877727</v>
-      </c>
+        <v>17.37169811320755</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="n">
+        <v>0.004035983490109473</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0.022356316076508</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>0.06191859676055975</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0.1143275010568631</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0.1583221138124134</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>0.1753971108635621</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>0.1619280347644893</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0.1281370924376426</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0.08872290194821135</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>0.05460646826066947</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>0.03024788052897153</v>
+      </c>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="inlineStr"/>
+      <c r="BA4" t="inlineStr"/>
+      <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr"/>
+      <c r="BG4" t="inlineStr"/>
+      <c r="BH4" t="inlineStr"/>
+      <c r="BI4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1653,41 +2243,97 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.9</v>
+        <v>15</v>
       </c>
       <c r="C5" t="n">
-        <v>0.05503533924501622</v>
+        <v>25</v>
       </c>
       <c r="D5" t="n">
-        <v>0.159602483810547</v>
+        <v>4.863461538461539</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2314236015252932</v>
+        <v>4.949894499460882</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2237094814744501</v>
+        <v>19.86346153846154</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1621893740689763</v>
+        <v>0.007176076426108307</v>
       </c>
       <c r="H5" t="n">
-        <v>0.09406983696000626</v>
+        <v>0.03552082122930442</v>
       </c>
       <c r="I5" t="n">
-        <v>0.04546708786400301</v>
+        <v>0.08791215880963363</v>
       </c>
       <c r="J5" t="n">
-        <v>0.01883636497222982</v>
+        <v>0.1450519704425123</v>
       </c>
       <c r="K5" t="n">
-        <v>0.006828182302433311</v>
+        <v>0.1794979876573386</v>
       </c>
       <c r="L5" t="n">
-        <v>0.002200192075228511</v>
+        <v>0.1776992203538715</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0006380557018162682</v>
-      </c>
+        <v>0.1465987322313526</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.1036640368999873</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.06414075575539463</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.03527666378943242</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.01746157640506424</v>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
+      <c r="BF5" t="inlineStr"/>
+      <c r="BG5" t="inlineStr"/>
+      <c r="BH5" t="inlineStr"/>
+      <c r="BI5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1696,41 +2342,97 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2.6</v>
+        <v>14</v>
       </c>
       <c r="C6" t="n">
-        <v>0.07428001934180856</v>
+        <v>24</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1931280502887023</v>
+        <v>5.14423076923077</v>
       </c>
       <c r="E6" t="n">
-        <v>0.251066465375313</v>
+        <v>5.270102960829012</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2175909366586045</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.141434108828093</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.07354573659060834</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.03186981918926361</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.01183736141315506</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.003847142459275395</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.001111396710457336</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.0002889631447189074</v>
-      </c>
+        <v>19.14423076923077</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="n">
+        <v>0.005244242027665033</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.02763769543730144</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.0728267502773064</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.1279348240879958</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.1685574238048214</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.1776629956527001</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.1560503799031744</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.1174859384523159</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.07739537401166567</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0.04532017663703868</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0.02388419970801513</v>
+      </c>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr"/>
+      <c r="BG6" t="inlineStr"/>
+      <c r="BH6" t="inlineStr"/>
+      <c r="BI6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1739,41 +2441,97 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2231302832612856</v>
+        <v>18</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3346954248919284</v>
+        <v>4.840384615384616</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2510215686689463</v>
+        <v>4.924083563192912</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1255107843344732</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.04706654412542743</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.01411996323762823</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.003529990809407058</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.000756426602015798</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.0001418299878779621</v>
-      </c>
-      <c r="L7" t="n">
-        <v>2.363833131299369e-05</v>
-      </c>
-      <c r="M7" t="n">
-        <v>3.545749696949053e-06</v>
-      </c>
+        <v>12.84038461538461</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="n">
+        <v>0.007360434843819656</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>0.03624339623240476</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>0.0892327558311361</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>0.1464631820955012</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>0.180299236892347</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0.1775617017675662</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>0.1457214428543725</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>0.1025063659377101</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>0.06309373895456452</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>0.03451987143628394</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>0.01699787315429383</v>
+      </c>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
+      <c r="BE7" t="inlineStr"/>
+      <c r="BF7" t="inlineStr"/>
+      <c r="BG7" t="inlineStr"/>
+      <c r="BH7" t="inlineStr"/>
+      <c r="BI7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1782,40 +2540,96 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.6</v>
+        <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>0.2018967249205256</v>
+        <v>17</v>
       </c>
       <c r="D8" t="n">
-        <v>0.323034759872841</v>
+        <v>4.740384615384615</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2584278078982729</v>
+        <v>4.813028767664369</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1378281642124122</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.05513126568496488</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.01764200501918876</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.00470453467178367</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.00107532221069341</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.0002150644421386821</v>
-      </c>
-      <c r="L8" t="n">
-        <v>3.823367860243238e-05</v>
-      </c>
-      <c r="M8" t="n">
-        <v>6.11738857638918e-06</v>
+        <v>11.74038461538462</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="n">
+        <v>0.008210330898792001</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>0.03951655880792955</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>0.09509716717083286</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>0.1525684671055354</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>0.1835791053043492</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>0.1767143029943838</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>0.1417551706616212</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>0.09746738776565068</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>0.05863916765314686</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>0.0313591112029433</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>0.01509323043481521</v>
       </c>
     </row>
   </sheetData>
@@ -1829,7 +2643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1847,51 +2661,97 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>annual_total_products</t>
+          <t>calendar_year</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7754.2</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>units_per_model_unit</t>
+          <t>annual_total_real_units</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.8</v>
+        <v>6257</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>average_daily_demand_in_model_units</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>11.80243531202435</v>
+          <t>annual_weekday_demands_real_units</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>[1059.3000000000002, 971.3000000000001, 920.7, 1032.9, 995.5000000000001, 667.7, 610.5]</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>max_noise</t>
+          <t>units_per_model_unit</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>max_noise_full_width_model_units</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>fit_lambda_to_centered_mean</t>
+        </is>
+      </c>
+      <c r="B7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>max_total_demand_column_K</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>D = lower_demand + Z, where Z is truncated Poisson on {0,...,max_noise}; E[D] matches the 2025 weekday mean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>If base demand is 15 and max_noise is 10, support is demand 10 through 20.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>